<commit_message>
Update Settings for ZeaMiC Data Comparison Proccessing.xlsx
</commit_message>
<xml_diff>
--- a/Maize Dataset Comparison/Settings for ZeaMiC Data Comparison Proccessing.xlsx
+++ b/Maize Dataset Comparison/Settings for ZeaMiC Data Comparison Proccessing.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kansas-my.sharepoint.com/personal/j853s117_home_ku_edu/Documents/Wagner Postdoc/!USDA_grant/Objective 1/Syncom Manuscript/CODE REPOSITORY/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kansas-my.sharepoint.com/personal/j853s117_home_ku_edu/Documents/GITHUB/ZeaMic_Culture_Collection/Maize Dataset Comparison/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="150" documentId="11_F25DC773A252ABDACC10487CB1D851865ADE58E9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0F3C78F2-DD5A-4AE3-934E-D9A429D5B3B7}"/>
+  <xr:revisionPtr revIDLastSave="151" documentId="11_F25DC773A252ABDACC10487CB1D851865ADE58E9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{13700A78-870F-4FD7-9A99-BB433212F87F}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -60,9 +60,6 @@
     <t>Hu et al. (2018)</t>
   </si>
   <si>
-    <t>Availiable as ASV from Author?</t>
-  </si>
-  <si>
     <t>Yes</t>
   </si>
   <si>
@@ -106,6 +103,9 @@
   </si>
   <si>
     <t>DADA2 maxEE for FWD Read</t>
+  </si>
+  <si>
+    <t>ASV table provided by Author?</t>
   </si>
 </sst>
 </file>
@@ -215,6 +215,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -499,28 +503,28 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D1" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E1" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="H1" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="I1" s="4" t="s">
         <v>24</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -528,26 +532,26 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -555,14 +559,14 @@
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C3" s="5"/>
       <c r="D3" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F3" s="5">
         <v>280</v>
@@ -582,16 +586,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D4" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="6" t="s">
         <v>15</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>16</v>
       </c>
       <c r="F4" s="5">
         <v>250</v>
@@ -611,26 +615,26 @@
         <v>4</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -638,14 +642,14 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F6" s="5">
         <v>220</v>
@@ -665,28 +669,28 @@
         <v>6</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F7" s="5">
         <v>250</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H7" s="5">
         <v>3</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
@@ -694,26 +698,26 @@
         <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -721,26 +725,26 @@
         <v>8</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C9" s="5"/>
       <c r="D9" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -748,26 +752,26 @@
         <v>9</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C10" s="5"/>
       <c r="D10" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -775,26 +779,26 @@
         <v>10</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C11" s="5"/>
       <c r="D11" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>